<commit_message>
feat(packing): 6D — packing estándar MADENAT (Forestal Andes), formato en lumber.ingestion.format y botón de descarga
</commit_message>
<xml_diff>
--- a/madenat_ingestion_engine/data/templates/PLANTILLA_PACKING_METRICO_ASERRADA.xlsx
+++ b/madenat_ingestion_engine/data/templates/PLANTILLA_PACKING_METRICO_ASERRADA.xlsx
@@ -538,26 +538,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MADENAT — PLANTILLA ESTÁNDAR DE PACKING LIST (SISTEMA MÉTRICO)</t>
+          <t>MADENAT — PACKING ESTÁNDAR (FORMATO FORESTAL ANDES)</t>
         </is>
       </c>
     </row>
@@ -579,7 +581,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>12345</t>
+          <t>40030</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -589,7 +591,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -600,6 +602,16 @@
       <c r="K2" s="3" t="inlineStr">
         <is>
           <t>OC-2026-001</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>PROVEEDOR</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>FORESTAL ANDES S.A.</t>
         </is>
       </c>
     </row>
@@ -621,42 +633,52 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
+          <t>SUBPRODUCTO</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
           <t>LOTE</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>ESPESOR</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>ANCHO</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>LARGO</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>FILAS</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>COLUMNAS</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>PIEZAS</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>VOLUMEN</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>PERFIL</t>
         </is>
       </c>
     </row>
@@ -676,29 +698,39 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>ETQ-001</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n">
+          <t>CLEAR</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>ETQ-ANDES-001</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="n">
         <v>38.1</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="G5" s="8" t="n">
         <v>170</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="H5" s="9" t="n">
         <v>4.05</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="I5" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="J5" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="K5" s="5" t="n">
         <v>150</v>
       </c>
-      <c r="K5" s="10" t="n">
+      <c r="L5" s="10" t="n">
         <v>3.886</v>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>packing_metrico_aserrada</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -712,34 +744,44 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>PINO ASERRADO SECO KD</t>
+          <t>PINO ASERRADO VERDE</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>ETQ-002</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>45</v>
+          <t>INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>ETQ-ARAUCO-002</t>
+        </is>
       </c>
       <c r="F6" s="8" t="n">
-        <v>125</v>
-      </c>
-      <c r="G6" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="H6" s="9" t="n">
         <v>3.6</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="I6" s="5" t="n">
-        <v>8</v>
-      </c>
       <c r="J6" s="5" t="n">
-        <v>160</v>
-      </c>
-      <c r="K6" s="10" t="n">
-        <v>3.24</v>
+        <v>6</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="L6" s="10" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>packing_metrico_aserrada</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -753,34 +795,44 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>PINO ASERRADO VERDE</t>
+          <t>PINO ASERRADO SECO KD</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>ETQ-003</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>25</v>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>ETQ-JCE-003</t>
+        </is>
       </c>
       <c r="F7" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="G7" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>125</v>
+      </c>
+      <c r="H7" s="9" t="n">
         <v>3.6</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="I7" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="J7" s="5" t="n">
-        <v>120</v>
-      </c>
-      <c r="K7" s="10" t="n">
-        <v>1.62</v>
+        <v>8</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="L7" s="10" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>packing_metrico_aserrada</t>
+        </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -794,40 +846,61 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>PINO ASERRADO VERDE</t>
+          <t>PINO CEPILLADO</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>ETQ-004</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="n">
+          <t>MILL RUN</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>ETQ-BYC-004</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="G8" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="H8" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="K8" s="5" t="n">
         <v>90</v>
       </c>
-      <c r="K8" s="10" t="n">
+      <c r="L8" s="10" t="n">
         <v>2.7</v>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>packing_metrico_aserrada</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="C5:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PINO ASERRADO SECO KD,PINO ASERRADO VERDE,PINO CEPILLADO,BLANKS CLEAR"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D5:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CLEAR,COL,INDUSTRIAL,MILL RUN,SELECTO,ESTANDAR"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M5:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"packing_metrico_aserrada,f1550,f5085,blanks,metric"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -838,17 +911,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="85" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>GUÍA DE LLENADO — SISTEMA DE INGESTA MADENAT (MÉTRICO)</t>
+          <t>GUÍA DE LLENADO — PACKING ESTÁNDAR MADENAT (FORESTAL ANDES)</t>
         </is>
       </c>
     </row>
@@ -859,7 +932,7 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>REGLAS GENERALES:</t>
+          <t>REGLAS GENERALES Y DECISIÓN DE OPERACIONES:</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr"/>
@@ -867,60 +940,60 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>1. Unidades</t>
+          <t>1. Formato Único</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>El sistema métrico aserrada asume Espesor en mm, Ancho en mm y Largo en metros (m).</t>
+          <t>Por decisión de Operaciones (respuesta Cristhian 8-oct), no se siguen adaptando lectores individuales para Arauco, JCE, BYC ni Fátima. Todos los proveedores deben ingresar a través de este Packing Estándar MADENAT.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>2. Volumen</t>
+          <t>2. Dimensiones Separadas</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>El volumen debe indicarse en metros cúbicos (m³). Fórmula típica: Espesor(mm)/1000 * Ancho(mm)/1000 * Largo(m) * Piezas.</t>
+          <t>El espesor debe venir en mm (columna ESPESOR), el ancho en mm (columna ANCHO) y el largo en metros (columna LARGO). JCE y Arauco deben desglosar escuadrías compuestas en estas 3 columnas.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>3. Paquetes / Lotes</t>
+          <t>3. Precisión de Volumen</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Cada fila representa un paquete físico (tarja). 'N°' identifica el paquete correlativo y 'LOTE' la etiqueta única del proveedor.</t>
+          <t>El packing manda sobre la guía. Si la guía viene con 2 decimales, el packing se redondea rigurosamente a 3 decimales (ej: 57,839556 m³ → 57,840 m³).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>4. Piezas</t>
+          <t>4. Listas Desplegables</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Debe coincidir con Filas * Columnas cuando el paquete sea regular, o con el recuento manual de piezas.</t>
+          <t>Utilice las opciones de las listas desplegables en PRODUCTO, SUBPRODUCTO y PERFIL para garantizar homologación directa en el inventario.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>5. Código / SKU</t>
+          <t>5. Trazabilidad de Tarjas</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Código de producto numérico o alfanumérico que identifica la escuadría y terminación.</t>
+          <t>Cada fila representa un paquete/tarja físico. El campo 'LOTE' preserva la etiqueta del proveedor de origen.</t>
         </is>
       </c>
     </row>
@@ -936,7 +1009,7 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>DESCRIPCIÓN Y EJEMPLO</t>
+          <t>DESCRIPCIÓN Y VALORES VÁLIDOS</t>
         </is>
       </c>
     </row>
@@ -948,7 +1021,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Identificador correlativo del paquete (Ej: 1, 2, 3...)</t>
+          <t>Número correlativo de tarja (Ej: 1, 2, 3...)</t>
         </is>
       </c>
     </row>
@@ -960,7 +1033,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Código de escuadría o SKU (Ej: 1000203040501)</t>
+          <t>Código SKU o referencia del producto (Ej: 1000203040501)</t>
         </is>
       </c>
     </row>
@@ -972,103 +1045,127 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Nombre descriptivo de la madera (Ej: PINO ASERRADO SECO KD)</t>
+          <t>Seleccione de la lista: PINO ASERRADO SECO KD, PINO ASERRADO VERDE, PINO CEPILLADO, BLANKS CLEAR</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>LOTE</t>
+          <t>SUBPRODUCTO</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>Número de etiqueta o lote asignado por el aserradero (Ej: ETQ-001)</t>
+          <t>Seleccione de la lista: CLEAR, COL, INDUSTRIAL, MILL RUN, SELECTO, ESTANDAR</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>ESPESOR</t>
+          <t>LOTE</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>Espesor en milímetros. Rango típico métrico: &gt;= 10 mm (Ej: 38.1, 45, 50)</t>
+          <t>Identificador único de la etiqueta o paquete (Ej: ETQ-001)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>ANCHO</t>
+          <t>ESPESOR</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Ancho en milímetros (Ej: 125, 150, 170)</t>
+          <t>Espesor nominal en mm (Ej: 25.0, 38.1, 45.0, 50.0)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>LARGO</t>
+          <t>ANCHO</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Largo nominal en metros (Ej: 3.60, 4.00, 4.05)</t>
+          <t>Ancho nominal en mm (Ej: 100.0, 125.0, 150.0, 170.0)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>FILAS</t>
+          <t>LARGO</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Capas verticales de madera en el paquete (Ej: 20, 25)</t>
+          <t>Largo nominal en metros (Ej: 3.20, 3.60, 4.00, 4.05)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>COLUMNAS</t>
+          <t>FILAS</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Piezas por capa a lo ancho (Ej: 6, 8)</t>
+          <t>Capas verticales de madera en el paquete (Ej: 20, 25)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>PIEZAS</t>
+          <t>COLUMNAS</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Número total de piezas contenidas en el paquete (Ej: 150)</t>
+          <t>Piezas por capa a lo ancho (Ej: 6, 8)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
+          <t>PIEZAS</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Total de piezas en el paquete (Ej: 120, 150, 160)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
           <t>VOLUMEN</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>Volumen cúbico total del paquete en m³ (Ej: 3.886)</t>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Volumen en m³ calculado a 3 decimales (Ej: 3.886)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>PERFIL</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Seleccione: packing_metrico_aserrada (estándar), f1550, f5085, blanks, metric</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ingestion): 6D — preservar plantilla métrica original y coexistencia con plantilla estándar MADENAT
</commit_message>
<xml_diff>
--- a/madenat_ingestion_engine/data/templates/PLANTILLA_PACKING_METRICO_ASERRADA.xlsx
+++ b/madenat_ingestion_engine/data/templates/PLANTILLA_PACKING_METRICO_ASERRADA.xlsx
@@ -538,28 +538,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MADENAT — PACKING ESTÁNDAR (FORMATO FORESTAL ANDES)</t>
+          <t>MADENAT — PLANTILLA ESTÁNDAR DE PACKING LIST (SISTEMA MÉTRICO)</t>
         </is>
       </c>
     </row>
@@ -581,7 +579,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>40030</t>
+          <t>12345</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -591,7 +589,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -602,16 +600,6 @@
       <c r="K2" s="3" t="inlineStr">
         <is>
           <t>OC-2026-001</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>PROVEEDOR</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>FORESTAL ANDES S.A.</t>
         </is>
       </c>
     </row>
@@ -633,52 +621,42 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>SUBPRODUCTO</t>
+          <t>LOTE</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>LOTE</t>
+          <t>ESPESOR</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>ESPESOR</t>
+          <t>ANCHO</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>ANCHO</t>
+          <t>LARGO</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>LARGO</t>
+          <t>FILAS</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>FILAS</t>
+          <t>COLUMNAS</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>COLUMNAS</t>
+          <t>PIEZAS</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>PIEZAS</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
           <t>VOLUMEN</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>PERFIL</t>
         </is>
       </c>
     </row>
@@ -698,39 +676,29 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>CLEAR</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>ETQ-ANDES-001</t>
-        </is>
+          <t>ETQ-001</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>38.1</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>38.1</v>
-      </c>
-      <c r="G5" s="8" t="n">
         <v>170</v>
       </c>
-      <c r="H5" s="9" t="n">
+      <c r="G5" s="9" t="n">
         <v>4.05</v>
       </c>
+      <c r="H5" s="5" t="n">
+        <v>25</v>
+      </c>
       <c r="I5" s="5" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K5" s="5" t="n">
         <v>150</v>
       </c>
-      <c r="L5" s="10" t="n">
+      <c r="K5" s="10" t="n">
         <v>3.886</v>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>packing_metrico_aserrada</t>
-        </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -744,44 +712,34 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>PINO ASERRADO VERDE</t>
+          <t>PINO ASERRADO SECO KD</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>INDUSTRIAL</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>ETQ-ARAUCO-002</t>
-        </is>
+          <t>ETQ-002</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>45</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="G6" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="H6" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="G6" s="9" t="n">
         <v>3.6</v>
       </c>
+      <c r="H6" s="5" t="n">
+        <v>20</v>
+      </c>
       <c r="I6" s="5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>120</v>
-      </c>
-      <c r="L6" s="10" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>packing_metrico_aserrada</t>
-        </is>
+        <v>160</v>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>3.24</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -795,44 +753,34 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>PINO ASERRADO SECO KD</t>
+          <t>PINO ASERRADO VERDE</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>COL</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>ETQ-JCE-003</t>
-        </is>
+          <t>ETQ-003</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>25</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="G7" s="8" t="n">
-        <v>125</v>
-      </c>
-      <c r="H7" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="G7" s="9" t="n">
         <v>3.6</v>
       </c>
+      <c r="H7" s="5" t="n">
+        <v>20</v>
+      </c>
       <c r="I7" s="5" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="K7" s="5" t="n">
-        <v>160</v>
-      </c>
-      <c r="L7" s="10" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="M7" s="6" t="inlineStr">
-        <is>
-          <t>packing_metrico_aserrada</t>
-        </is>
+        <v>120</v>
+      </c>
+      <c r="K7" s="10" t="n">
+        <v>1.62</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -846,61 +794,40 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>PINO CEPILLADO</t>
+          <t>PINO ASERRADO VERDE</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>MILL RUN</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>ETQ-BYC-004</t>
-        </is>
+          <t>ETQ-004</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>50</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="G8" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="G8" s="9" t="n">
         <v>4</v>
       </c>
+      <c r="H8" s="5" t="n">
+        <v>15</v>
+      </c>
       <c r="I8" s="5" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K8" s="5" t="n">
         <v>90</v>
       </c>
-      <c r="L8" s="10" t="n">
+      <c r="K8" s="10" t="n">
         <v>2.7</v>
-      </c>
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>packing_metrico_aserrada</t>
-        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation sqref="C5:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PINO ASERRADO SECO KD,PINO ASERRADO VERDE,PINO CEPILLADO,BLANKS CLEAR"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D5:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"CLEAR,COL,INDUSTRIAL,MILL RUN,SELECTO,ESTANDAR"</formula1>
-    </dataValidation>
-    <dataValidation sqref="M5:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"packing_metrico_aserrada,f1550,f5085,blanks,metric"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -911,17 +838,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="85" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>GUÍA DE LLENADO — PACKING ESTÁNDAR MADENAT (FORESTAL ANDES)</t>
+          <t>GUÍA DE LLENADO — SISTEMA DE INGESTA MADENAT (MÉTRICO)</t>
         </is>
       </c>
     </row>
@@ -932,7 +859,7 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>REGLAS GENERALES Y DECISIÓN DE OPERACIONES:</t>
+          <t>REGLAS GENERALES:</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr"/>
@@ -940,60 +867,60 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>1. Formato Único</t>
+          <t>1. Unidades</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Por decisión de Operaciones (respuesta Cristhian 8-oct), no se siguen adaptando lectores individuales para Arauco, JCE, BYC ni Fátima. Todos los proveedores deben ingresar a través de este Packing Estándar MADENAT.</t>
+          <t>El sistema métrico aserrada asume Espesor en mm, Ancho en mm y Largo en metros (m).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>2. Dimensiones Separadas</t>
+          <t>2. Volumen</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>El espesor debe venir en mm (columna ESPESOR), el ancho en mm (columna ANCHO) y el largo en metros (columna LARGO). JCE y Arauco deben desglosar escuadrías compuestas en estas 3 columnas.</t>
+          <t>El volumen debe indicarse en metros cúbicos (m³). Fórmula típica: Espesor(mm)/1000 * Ancho(mm)/1000 * Largo(m) * Piezas.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>3. Precisión de Volumen</t>
+          <t>3. Paquetes / Lotes</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>El packing manda sobre la guía. Si la guía viene con 2 decimales, el packing se redondea rigurosamente a 3 decimales (ej: 57,839556 m³ → 57,840 m³).</t>
+          <t>Cada fila representa un paquete físico (tarja). 'N°' identifica el paquete correlativo y 'LOTE' la etiqueta única del proveedor.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>4. Listas Desplegables</t>
+          <t>4. Piezas</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Utilice las opciones de las listas desplegables en PRODUCTO, SUBPRODUCTO y PERFIL para garantizar homologación directa en el inventario.</t>
+          <t>Debe coincidir con Filas * Columnas cuando el paquete sea regular, o con el recuento manual de piezas.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>5. Trazabilidad de Tarjas</t>
+          <t>5. Código / SKU</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Cada fila representa un paquete/tarja físico. El campo 'LOTE' preserva la etiqueta del proveedor de origen.</t>
+          <t>Código de producto numérico o alfanumérico que identifica la escuadría y terminación.</t>
         </is>
       </c>
     </row>
@@ -1009,7 +936,7 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>DESCRIPCIÓN Y VALORES VÁLIDOS</t>
+          <t>DESCRIPCIÓN Y EJEMPLO</t>
         </is>
       </c>
     </row>
@@ -1021,7 +948,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Número correlativo de tarja (Ej: 1, 2, 3...)</t>
+          <t>Identificador correlativo del paquete (Ej: 1, 2, 3...)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +960,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Código SKU o referencia del producto (Ej: 1000203040501)</t>
+          <t>Código de escuadría o SKU (Ej: 1000203040501)</t>
         </is>
       </c>
     </row>
@@ -1045,127 +972,103 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Seleccione de la lista: PINO ASERRADO SECO KD, PINO ASERRADO VERDE, PINO CEPILLADO, BLANKS CLEAR</t>
+          <t>Nombre descriptivo de la madera (Ej: PINO ASERRADO SECO KD)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>SUBPRODUCTO</t>
+          <t>LOTE</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>Seleccione de la lista: CLEAR, COL, INDUSTRIAL, MILL RUN, SELECTO, ESTANDAR</t>
+          <t>Número de etiqueta o lote asignado por el aserradero (Ej: ETQ-001)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>LOTE</t>
+          <t>ESPESOR</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>Identificador único de la etiqueta o paquete (Ej: ETQ-001)</t>
+          <t>Espesor en milímetros. Rango típico métrico: &gt;= 10 mm (Ej: 38.1, 45, 50)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>ESPESOR</t>
+          <t>ANCHO</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Espesor nominal en mm (Ej: 25.0, 38.1, 45.0, 50.0)</t>
+          <t>Ancho en milímetros (Ej: 125, 150, 170)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>ANCHO</t>
+          <t>LARGO</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Ancho nominal en mm (Ej: 100.0, 125.0, 150.0, 170.0)</t>
+          <t>Largo nominal en metros (Ej: 3.60, 4.00, 4.05)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>LARGO</t>
+          <t>FILAS</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Largo nominal en metros (Ej: 3.20, 3.60, 4.00, 4.05)</t>
+          <t>Capas verticales de madera en el paquete (Ej: 20, 25)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>FILAS</t>
+          <t>COLUMNAS</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Capas verticales de madera en el paquete (Ej: 20, 25)</t>
+          <t>Piezas por capa a lo ancho (Ej: 6, 8)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>COLUMNAS</t>
+          <t>PIEZAS</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Piezas por capa a lo ancho (Ej: 6, 8)</t>
+          <t>Número total de piezas contenidas en el paquete (Ej: 150)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>PIEZAS</t>
+          <t>VOLUMEN</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Total de piezas en el paquete (Ej: 120, 150, 160)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>VOLUMEN</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>Volumen en m³ calculado a 3 decimales (Ej: 3.886)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>PERFIL</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Seleccione: packing_metrico_aserrada (estándar), f1550, f5085, blanks, metric</t>
+          <t>Volumen cúbico total del paquete en m³ (Ej: 3.886)</t>
         </is>
       </c>
     </row>

</xml_diff>